<commit_message>
v1.7.0: investimentos edicao/exclusao, cartao ajustes, tudo finalizado
</commit_message>
<xml_diff>
--- a/gastosset.xlsx
+++ b/gastosset.xlsx
@@ -1,41 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Darci\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Darci\Documents\Darci\GitHub\Gastos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6273A86B-EB5D-4798-8097-3477279D61A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70AAF1DF-C0B0-41AC-B28B-6368738850D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B3C48F16-DB74-4FA7-B964-47D0E2A6E77E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Gastos" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
   <si>
     <t>Sicredi</t>
   </si>
@@ -145,7 +135,13 @@
     <t>Parcelado</t>
   </si>
   <si>
-    <t>Saidas</t>
+    <t>Vale</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 09/12</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 08/12</t>
   </si>
 </sst>
 </file>
@@ -533,28 +529,58 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>20</v>
+      </c>
+      <c r="B2">
+        <v>1600</v>
+      </c>
+      <c r="D2" s="1">
+        <v>46266</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="B3">
-        <v>2200</v>
+        <v>760</v>
+      </c>
+      <c r="D3" s="1">
+        <v>46266</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4">
+        <v>1500</v>
+      </c>
+      <c r="D4" s="1">
+        <v>46280</v>
+      </c>
+      <c r="E4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B4">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>36</v>
+      <c r="B5">
+        <v>650</v>
+      </c>
+      <c r="D5" s="1">
+        <v>46280</v>
+      </c>
+      <c r="E5" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -581,6 +607,9 @@
       <c r="D8" s="1">
         <v>46254</v>
       </c>
+      <c r="E8" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -592,6 +621,9 @@
       <c r="D9" s="1">
         <v>46285</v>
       </c>
+      <c r="E9" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -603,6 +635,9 @@
       <c r="D10" s="1">
         <v>46285</v>
       </c>
+      <c r="E10" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -722,7 +757,7 @@
       </c>
       <c r="B19">
         <f>SUM(B1:B18)</f>
-        <v>2470</v>
+        <v>4510</v>
       </c>
       <c r="C19">
         <f>SUM(C1:C18)</f>

</xml_diff>